<commit_message>
Added logging functionality: log4j2
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="39">
   <si>
     <t>Name</t>
   </si>
@@ -807,7 +807,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>34</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -815,7 +815,7 @@
         <v>2.0</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>35</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -823,7 +823,7 @@
         <v>3.0</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>36</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -831,7 +831,7 @@
         <v>4.0</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -847,7 +847,7 @@
         <v>6.0</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>37</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
@@ -855,7 +855,7 @@
         <v>7.0</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>38</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Added more system info in Extent Report
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="39">
   <si>
     <t>Name</t>
   </si>
@@ -807,7 +807,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>17</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
@@ -815,7 +815,7 @@
         <v>2.0</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>18</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4">
@@ -823,7 +823,7 @@
         <v>3.0</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>19</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
@@ -831,7 +831,7 @@
         <v>4.0</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -847,7 +847,7 @@
         <v>6.0</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>22</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8">
@@ -855,7 +855,7 @@
         <v>7.0</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>23</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9">

</xml_diff>